<commit_message>
feat: tela de perfil adicionada
</commit_message>
<xml_diff>
--- a/public/modelo-cadastro-usuarios-acervo.xlsx
+++ b/public/modelo-cadastro-usuarios-acervo.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alunos" sheetId="1" r:id="Rb3a64ee56de440a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Professores" sheetId="2" r:id="R2da2178a4bb64215"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instruções" sheetId="3" r:id="Rcb37b73161184ea0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alunos" sheetId="1" r:id="R4f984441dc774a64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Professores" sheetId="2" r:id="R444770ea69b34802"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instruções" sheetId="3" r:id="R613534494a06498d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -318,7 +318,7 @@
         <x:v>Nome Aluno</x:v>
       </x:c>
       <x:c r="D1" s="6" t="str">
-        <x:v>E-mail Institucional</x:v>
+        <x:v>E-mail</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -343,7 +343,7 @@
         <x:v>Professores DSM</x:v>
       </x:c>
       <x:c r="C1" s="6" t="str">
-        <x:v>E-mail Institucional</x:v>
+        <x:v>E-mail</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -380,7 +380,7 @@
         <x:v>Alunos</x:v>
       </x:c>
       <x:c r="B3" s="16" t="str">
-        <x:v>Curso, RA, Nome Aluno e E-mail Institucional são os cabeçalhos esperados.</x:v>
+        <x:v>Curso, RA, Nome Aluno e E-mail são os cabeçalhos esperados.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="34" customHeight="1">
@@ -388,7 +388,7 @@
         <x:v>Professores</x:v>
       </x:c>
       <x:c r="B4" s="16" t="str">
-        <x:v>Matrícula, Professores DSM e E-mail Institucional são os cabeçalhos esperados.</x:v>
+        <x:v>Matrícula, Professores DSM e E-mail são os cabeçalhos esperados.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
@@ -412,7 +412,7 @@
         <x:v>Privacidade</x:v>
       </x:c>
       <x:c r="B7" s="16" t="str">
-        <x:v>Não publique planilhas preenchidas com nome, RA/matrícula ou e-mail institucional. Acesse e use a planilha real apenas no painel administrativo.</x:v>
+        <x:v>Não publique planilhas preenchidas com dados pessoais. Use a planilha real apenas no painel administrativo.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>